<commit_message>
Sub-agrupacion estricta de vigas por longitud + condicion de apoyo (12 VC + 16 VR): Excel, memoria (tablas 61/62) y planos actualizados
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Diseno-Estructural-Calculos.xlsx
@@ -90,8 +90,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -143,7 +143,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VC-1 a VC-9 (por longitud)</t>
+          <t xml:space="preserve">VC agrupadas por LONGITUD + CONDICIÓN DE APOYO</t>
         </is>
       </c>
     </row>
@@ -155,7 +155,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VR-1 a VR-11 (por longitud)</t>
+          <t xml:space="preserve">VR agrupadas por LONGITUD + CONDICIÓN DE APOYO</t>
         </is>
       </c>
     </row>
@@ -167,7 +167,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coeficientes NSR-10 C.8.3.3 según apoyo</t>
+          <t xml:space="preserve">Coeficientes NSR-10 C.8.3.3 según apoyo (1EC/2EC/V)</t>
         </is>
       </c>
     </row>
@@ -190,11 +190,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -264,7 +264,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. IRREGULARIDADES EN PLANTA  →  φp</t>
+          <t xml:space="preserve">2. IRREGULARIDADES EN PLANTA → φp</t>
         </is>
       </c>
     </row>
@@ -397,7 +397,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. IRREGULARIDADES EN ALTURA  →  φa</t>
+          <t xml:space="preserve">3. IRREGULARIDADES EN ALTURA → φa</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. REDUNDANCIA  →  φr</t>
+          <t xml:space="preserve">4. REDUNDANCIA → φr</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.0 · 1.00 · 1.00 · 1.00</t>
+          <t xml:space="preserve">5.0·1.00·1.00·1.00</t>
         </is>
       </c>
       <c r="C27" s="0"/>
@@ -585,35 +585,40 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIGAS DE CARGA VC — agrupadas por longitud</t>
+          <t xml:space="preserve">VIGAS DE CARGA VC — agrupadas por longitud + condición de apoyo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sección 0.30×0.40 m · d=342.6 mm · diseño con la mayor solicitación de cada grupo (sismo ÷ R=5)</t>
+          <t xml:space="preserve">Sección 0.30×0.40 m · d=342.6 mm · sismo ÷ R=5</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criterio del profesor: se agrupan vigas con la MISMA longitud Y la MISMA condición de apoyo; cada grupo se diseña con su mayor solicitación.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -628,45 +633,50 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Cond. apoyo</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Nº vigas</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Mu⁻ (kN·m)</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Mu⁺ (kN·m)</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Vu (kN)</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Tu (kN·m)</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ref. superior</t>
-        </is>
-      </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ref. inferior</t>
+          <t xml:space="preserve">Ref. sup.</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ref. inf.</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">φVc (kN)</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="L4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Estribo Nº3</t>
         </is>
@@ -681,35 +691,40 @@
       <c r="B5" s="3">
         <v>2.5</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D5" s="3">
         <v>20</v>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="3">
         <v>-10.4</v>
       </c>
-      <c r="E5" s="3">
+      <c r="F5" s="3">
         <v>4.0</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <v>14.2</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>1.9</v>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2 Nº5</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2 Nº5</t>
         </is>
       </c>
-      <c r="J5" s="3">
+      <c r="K5" s="3">
         <v>69.3</v>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -724,35 +739,40 @@
       <c r="B6" s="3">
         <v>2.6</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D6" s="3">
         <v>20</v>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="3">
         <v>-6.9</v>
       </c>
-      <c r="E6" s="3">
+      <c r="F6" s="3">
         <v>2.3</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>12.0</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>0.3</v>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2 Nº5</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2 Nº5</t>
         </is>
       </c>
-      <c r="J6" s="3">
+      <c r="K6" s="3">
         <v>69.3</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -767,35 +787,40 @@
       <c r="B7" s="3">
         <v>2.65</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D7" s="3">
         <v>20</v>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="3">
         <v>-118.8</v>
       </c>
-      <c r="E7" s="3">
+      <c r="F7" s="3">
         <v>102.8</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="3">
         <v>88.3</v>
       </c>
-      <c r="G7" s="3">
+      <c r="H7" s="3">
         <v>0</v>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">6 Nº5</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Nº5</t>
         </is>
       </c>
-      <c r="J7" s="3">
+      <c r="K7" s="3">
         <v>69.3</v>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -810,35 +835,40 @@
       <c r="B8" s="3">
         <v>3.75</v>
       </c>
-      <c r="C8" s="3">
-        <v>40</v>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D8" s="3">
+        <v>28</v>
+      </c>
+      <c r="E8" s="3">
         <v>-106.0</v>
       </c>
-      <c r="E8" s="3">
+      <c r="F8" s="3">
         <v>89.6</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <v>64.9</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="3">
         <v>0</v>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Nº5</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
-      <c r="J8" s="3">
+      <c r="K8" s="3">
         <v>69.3</v>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -851,37 +881,42 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <v>3.81</v>
-      </c>
-      <c r="C9" s="3">
-        <v>20</v>
+        <v>3.75</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
       </c>
       <c r="D9" s="3">
-        <v>-113.9</v>
+        <v>12</v>
       </c>
       <c r="E9" s="3">
-        <v>81.1</v>
+        <v>-25.0</v>
       </c>
       <c r="F9" s="3">
-        <v>73.5</v>
+        <v>16.5</v>
       </c>
       <c r="G9" s="3">
-        <v>6.9</v>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Nº5</t>
-        </is>
+        <v>21.7</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-      <c r="J9" s="3">
+          <t xml:space="preserve">2 Nº5</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº5</t>
+        </is>
+      </c>
+      <c r="K9" s="3">
         <v>69.3</v>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -894,37 +929,42 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <v>3.85</v>
-      </c>
-      <c r="C10" s="3">
-        <v>60</v>
+        <v>3.81</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D10" s="3">
-        <v>-121.6</v>
+        <v>16</v>
       </c>
       <c r="E10" s="3">
-        <v>93.3</v>
+        <v>-113.9</v>
       </c>
       <c r="F10" s="3">
-        <v>77.9</v>
+        <v>81.1</v>
       </c>
       <c r="G10" s="3">
-        <v>0</v>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 Nº5</t>
-        </is>
+        <v>73.5</v>
+      </c>
+      <c r="H10" s="3">
+        <v>6.9</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
-      <c r="J10" s="3">
+      <c r="K10" s="3">
         <v>69.3</v>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -937,37 +977,42 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <v>3.9</v>
-      </c>
-      <c r="C11" s="3">
-        <v>40</v>
+        <v>3.81</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
       </c>
       <c r="D11" s="3">
-        <v>-128.9</v>
+        <v>4</v>
       </c>
       <c r="E11" s="3">
-        <v>90.7</v>
+        <v>-105.7</v>
       </c>
       <c r="F11" s="3">
-        <v>91.9</v>
+        <v>74.2</v>
       </c>
       <c r="G11" s="3">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 Nº5</t>
-        </is>
+        <v>68.4</v>
+      </c>
+      <c r="H11" s="3">
+        <v>6.5</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
-      <c r="J11" s="3">
+      <c r="K11" s="3">
         <v>69.3</v>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -980,37 +1025,42 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="C12" s="3">
-        <v>40</v>
+        <v>3.85</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
       </c>
       <c r="D12" s="3">
-        <v>-104.0</v>
+        <v>60</v>
       </c>
       <c r="E12" s="3">
-        <v>87.2</v>
+        <v>-121.6</v>
       </c>
       <c r="F12" s="3">
-        <v>60.1</v>
+        <v>93.3</v>
       </c>
       <c r="G12" s="3">
+        <v>77.9</v>
+      </c>
+      <c r="H12" s="3">
         <v>0</v>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Nº5</t>
-        </is>
-      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">6 Nº5</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
-      <c r="J12" s="3">
+      <c r="K12" s="3">
         <v>69.3</v>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1023,37 +1073,186 @@
         </is>
       </c>
       <c r="B13" s="3">
+        <v>3.9</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D13" s="3">
+        <v>40</v>
+      </c>
+      <c r="E13" s="3">
+        <v>-128.9</v>
+      </c>
+      <c r="F13" s="3">
+        <v>90.7</v>
+      </c>
+      <c r="G13" s="3">
+        <v>91.9</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 Nº5</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
+      </c>
+      <c r="K13" s="3">
+        <v>69.3</v>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VC-10</t>
+        </is>
+      </c>
+      <c r="B14" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D14" s="3">
+        <v>40</v>
+      </c>
+      <c r="E14" s="3">
+        <v>-104.0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>87.2</v>
+      </c>
+      <c r="G14" s="3">
+        <v>60.1</v>
+      </c>
+      <c r="H14" s="3">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
+      </c>
+      <c r="K14" s="3">
+        <v>69.3</v>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VC-11</t>
+        </is>
+      </c>
+      <c r="B15" s="3">
         <v>5.1</v>
       </c>
-      <c r="C13" s="3">
-        <v>20</v>
-      </c>
-      <c r="D13" s="3">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D15" s="3">
+        <v>16</v>
+      </c>
+      <c r="E15" s="3">
         <v>-97.5</v>
       </c>
-      <c r="E13" s="3">
+      <c r="F15" s="3">
         <v>71.0</v>
       </c>
-      <c r="F13" s="3">
+      <c r="G15" s="3">
         <v>50.0</v>
       </c>
-      <c r="G13" s="3">
+      <c r="H15" s="3">
         <v>0</v>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Nº5</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J13" s="3">
+      <c r="K15" s="3">
         <v>69.3</v>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VC-12</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <v>5.1</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D16" s="3">
+        <v>4</v>
+      </c>
+      <c r="E16" s="3">
+        <v>-93.3</v>
+      </c>
+      <c r="F16" s="3">
+        <v>68.1</v>
+      </c>
+      <c r="G16" s="3">
+        <v>48.5</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K16" s="3">
+        <v>69.3</v>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1066,35 +1265,40 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIGAS DE RIGIDEZ VR — agrupadas por longitud</t>
+          <t xml:space="preserve">VIGAS DE RIGIDEZ VR — agrupadas por longitud + condición de apoyo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sección 0.35×0.40 m · d=342.6 mm · diseño con la mayor solicitación de cada grupo (sismo ÷ R=5)</t>
+          <t xml:space="preserve">Sección 0.35×0.40 m · d=342.6 mm · sismo ÷ R=5</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criterio del profesor: se agrupan vigas con la MISMA longitud Y la MISMA condición de apoyo; cada grupo se diseña con su mayor solicitación.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1109,45 +1313,50 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Cond. apoyo</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Nº vigas</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Mu⁻ (kN·m)</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Mu⁺ (kN·m)</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Vu (kN)</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Tu (kN·m)</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ref. superior</t>
-        </is>
-      </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ref. inferior</t>
+          <t xml:space="preserve">Ref. sup.</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ref. inf.</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">φVc (kN)</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="L4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Estribo Nº3</t>
         </is>
@@ -1162,35 +1371,40 @@
       <c r="B5" s="3">
         <v>1.5</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D5" s="3">
         <v>30</v>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="3">
         <v>-57.9</v>
       </c>
-      <c r="E5" s="3">
+      <c r="F5" s="3">
         <v>55.0</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <v>81.2</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>25.7</v>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J5" s="3">
+      <c r="K5" s="3">
         <v>80.9</v>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1205,35 +1419,40 @@
       <c r="B6" s="3">
         <v>2.5</v>
       </c>
-      <c r="C6" s="3">
-        <v>50</v>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D6" s="3">
+        <v>32</v>
+      </c>
+      <c r="E6" s="3">
         <v>-32.4</v>
       </c>
-      <c r="E6" s="3">
+      <c r="F6" s="3">
         <v>11.0</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>56.9</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>0.6</v>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J6" s="3">
+      <c r="K6" s="3">
         <v>80.9</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1246,37 +1465,42 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <v>2.6</v>
-      </c>
-      <c r="C7" s="3">
-        <v>90</v>
+        <v>2.5</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
       </c>
       <c r="D7" s="3">
-        <v>-97.1</v>
+        <v>18</v>
       </c>
       <c r="E7" s="3">
-        <v>86.8</v>
+        <v>-27.2</v>
       </c>
       <c r="F7" s="3">
-        <v>154.3</v>
+        <v>10.3</v>
       </c>
       <c r="G7" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Nº5</t>
-        </is>
+        <v>54.8</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0.4</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-      <c r="J7" s="3">
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K7" s="3">
         <v>80.9</v>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1289,37 +1513,42 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="C8" s="3">
-        <v>15</v>
+        <v>2.6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D8" s="3">
-        <v>-81.1</v>
+        <v>30</v>
       </c>
       <c r="E8" s="3">
-        <v>42.6</v>
+        <v>-97.1</v>
       </c>
       <c r="F8" s="3">
-        <v>88.7</v>
+        <v>86.8</v>
       </c>
       <c r="G8" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
+        <v>154.3</v>
+      </c>
+      <c r="H8" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 Nº5</t>
-        </is>
-      </c>
-      <c r="J8" s="3">
+      <c r="K8" s="3">
         <v>80.9</v>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1332,37 +1561,42 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <v>2.8</v>
-      </c>
-      <c r="C9" s="3">
-        <v>15</v>
+        <v>2.6</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
       </c>
       <c r="D9" s="3">
-        <v>-78.8</v>
+        <v>60</v>
       </c>
       <c r="E9" s="3">
-        <v>37.4</v>
+        <v>-28.9</v>
       </c>
       <c r="F9" s="3">
-        <v>85.9</v>
+        <v>14.4</v>
       </c>
       <c r="G9" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
+        <v>56.0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>6.4</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K9" s="3">
         <v>80.9</v>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1375,37 +1609,42 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <v>2.95</v>
-      </c>
-      <c r="C10" s="3">
-        <v>10</v>
+        <v>2.7</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D10" s="3">
-        <v>-56.0</v>
+        <v>15</v>
       </c>
       <c r="E10" s="3">
-        <v>45.8</v>
+        <v>-81.1</v>
       </c>
       <c r="F10" s="3">
-        <v>95.4</v>
+        <v>42.6</v>
       </c>
       <c r="G10" s="3">
-        <v>1.7</v>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
+        <v>88.7</v>
+      </c>
+      <c r="H10" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 Nº5</t>
-        </is>
-      </c>
-      <c r="J10" s="3">
+      <c r="K10" s="3">
         <v>80.9</v>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1418,37 +1657,42 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <v>3.3</v>
-      </c>
-      <c r="C11" s="3">
-        <v>10</v>
+        <v>2.8</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D11" s="3">
-        <v>-39.0</v>
+        <v>15</v>
       </c>
       <c r="E11" s="3">
-        <v>14.9</v>
+        <v>-78.8</v>
       </c>
       <c r="F11" s="3">
-        <v>58.4</v>
+        <v>37.4</v>
       </c>
       <c r="G11" s="3">
-        <v>1.1</v>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
+        <v>85.9</v>
+      </c>
+      <c r="H11" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 Nº5</t>
-        </is>
-      </c>
-      <c r="J11" s="3">
+      <c r="K11" s="3">
         <v>80.9</v>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1461,37 +1705,42 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <v>3.65</v>
-      </c>
-      <c r="C12" s="3">
-        <v>40</v>
+        <v>2.95</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D12" s="3">
-        <v>-46.7</v>
+        <v>10</v>
       </c>
       <c r="E12" s="3">
-        <v>35.0</v>
+        <v>-56.0</v>
       </c>
       <c r="F12" s="3">
-        <v>110.6</v>
+        <v>45.8</v>
       </c>
       <c r="G12" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
+        <v>95.4</v>
+      </c>
+      <c r="H12" s="3">
+        <v>1.7</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J12" s="3">
+      <c r="K12" s="3">
         <v>80.9</v>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1504,37 +1753,42 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="C13" s="3">
-        <v>30</v>
+        <v>3.3</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
       </c>
       <c r="D13" s="3">
-        <v>-65.2</v>
+        <v>6</v>
       </c>
       <c r="E13" s="3">
-        <v>27.5</v>
+        <v>-39.0</v>
       </c>
       <c r="F13" s="3">
-        <v>85.2</v>
+        <v>14.9</v>
       </c>
       <c r="G13" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
+        <v>58.4</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J13" s="3">
+      <c r="K13" s="3">
         <v>80.9</v>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1547,37 +1801,42 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <v>4.18</v>
-      </c>
-      <c r="C14" s="3">
-        <v>20</v>
+        <v>3.3</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
       </c>
       <c r="D14" s="3">
-        <v>-78.0</v>
+        <v>4</v>
       </c>
       <c r="E14" s="3">
-        <v>26.2</v>
+        <v>-36.9</v>
       </c>
       <c r="F14" s="3">
-        <v>79.2</v>
+        <v>14.7</v>
       </c>
       <c r="G14" s="3">
-        <v>0.8</v>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
+        <v>57.3</v>
+      </c>
+      <c r="H14" s="3">
+        <v>1.1</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J14" s="3">
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K14" s="3">
         <v>80.9</v>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1590,37 +1849,282 @@
         </is>
       </c>
       <c r="B15" s="3">
+        <v>3.65</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D15" s="3">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3">
+        <v>-38.1</v>
+      </c>
+      <c r="F15" s="3">
+        <v>34.6</v>
+      </c>
+      <c r="G15" s="3">
+        <v>109.7</v>
+      </c>
+      <c r="H15" s="3">
+        <v>5.7</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K15" s="3">
+        <v>80.9</v>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VR-12</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <v>3.65</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D16" s="3">
+        <v>28</v>
+      </c>
+      <c r="E16" s="3">
+        <v>-46.7</v>
+      </c>
+      <c r="F16" s="3">
+        <v>35.0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>110.6</v>
+      </c>
+      <c r="H16" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K16" s="3">
+        <v>80.9</v>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VR-13</t>
+        </is>
+      </c>
+      <c r="B17" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="D17" s="3">
+        <v>8</v>
+      </c>
+      <c r="E17" s="3">
+        <v>-65.2</v>
+      </c>
+      <c r="F17" s="3">
+        <v>22.8</v>
+      </c>
+      <c r="G17" s="3">
+        <v>74.0</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K17" s="3">
+        <v>80.9</v>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VR-14</t>
+        </is>
+      </c>
+      <c r="B18" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D18" s="3">
+        <v>22</v>
+      </c>
+      <c r="E18" s="3">
+        <v>-60.9</v>
+      </c>
+      <c r="F18" s="3">
+        <v>27.5</v>
+      </c>
+      <c r="G18" s="3">
+        <v>85.2</v>
+      </c>
+      <c r="H18" s="3">
         <v>5.5</v>
       </c>
-      <c r="C15" s="3">
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K18" s="3">
+        <v>80.9</v>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VR-15</t>
+        </is>
+      </c>
+      <c r="B19" s="3">
+        <v>4.18</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D19" s="3">
+        <v>20</v>
+      </c>
+      <c r="E19" s="3">
+        <v>-78.0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>26.2</v>
+      </c>
+      <c r="G19" s="3">
+        <v>79.2</v>
+      </c>
+      <c r="H19" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
+      </c>
+      <c r="K19" s="3">
+        <v>80.9</v>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VR-16</t>
+        </is>
+      </c>
+      <c r="B20" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interior</t>
+        </is>
+      </c>
+      <c r="D20" s="3">
         <v>2</v>
       </c>
-      <c r="D15" s="3">
+      <c r="E20" s="3">
         <v>-103.8</v>
       </c>
-      <c r="E15" s="3">
+      <c r="F20" s="3">
         <v>50.6</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G20" s="3">
         <v>113.3</v>
       </c>
-      <c r="G15" s="3">
+      <c r="H20" s="3">
         <v>0.0</v>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">5 Nº5</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
-      <c r="J15" s="3">
+      <c r="K20" s="3">
         <v>80.9</v>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
@@ -1633,26 +2137,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DISEÑO DE VIGUETAS — momentos por coeficientes NSR-10 C.8.3.3</t>
+          <t xml:space="preserve">DISEÑO DE VIGUETAS — coeficientes NSR-10 C.8.3.3 según apoyo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Losa aligerada 1 dirección · nervio 0.15×0.34 · loseta 0.06 · sep 0.80 · d=304 mm · As_min=152 mm²</t>
+          <t xml:space="preserve">Nervio 0.15×0.34 + loseta 0.06 · sep 0.80 · d=304 mm · As_min=152 mm²</t>
         </is>
       </c>
     </row>
@@ -1660,87 +2164,102 @@
       <c r="A3" s="0"/>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Coeficiente según tipo de apoyo de cada vano:</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Código</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apoyo</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M⁺</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M⁻</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Código</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apoyo</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M⁺</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M⁻</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1EC</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vano extremo</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu·ln²/14</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1er apoyo int.: wu·ln²/10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1EC</t>
+          <t xml:space="preserve">2EC</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vano extremo (1 extremo continuo)</t>
+          <t xml:space="preserve">Vano interior</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">wu·ln²/14</t>
+          <t xml:space="preserve">wu·ln²/16</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1er apoyo int.: wu·ln²/10</t>
+          <t xml:space="preserve">apoyos: wu·ln²/11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2EC</t>
+          <t xml:space="preserve">(ext.)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vano interior (2 extremos continuos)</t>
+          <t xml:space="preserve">Apoyo exterior monolítico</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">wu·ln²/16</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">apoyos: wu·ln²/11</t>
+          <t xml:space="preserve">wu·ln²/24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">(ext.)</t>
+          <t xml:space="preserve">V</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apoyo exterior monolítico</t>
+          <t xml:space="preserve">Voladizo</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1750,99 +2269,126 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">wu·ln²/24</t>
+          <t xml:space="preserve">wu·L²/2</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">V</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Voladizo</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">wu·L²/2</t>
-        </is>
-      </c>
+      <c r="A9" s="0"/>
     </row>
     <row r="10">
-      <c r="A10" s="0"/>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caso</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ln (m)</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wu (kN/m)</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M⁻</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M⁺</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As req</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refuerzo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Casos gobernantes:</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrepiso vano extremo 1EC</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <v>4.75</v>
+      </c>
+      <c r="C11" s="3">
+        <v>9.06</v>
+      </c>
+      <c r="D11" s="3">
+        <v>20.4</v>
+      </c>
+      <c r="E11" s="3">
+        <v>14.6</v>
+      </c>
+      <c r="F11" s="3">
+        <v>185</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº4</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Caso</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ln (m)</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">wu (kN/m)</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M⁻</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M⁺</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">As req</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Refuerzo</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cubierta vano 1EC (terraza)</t>
+        </is>
+      </c>
+      <c r="B12" s="3">
+        <v>4.75</v>
+      </c>
+      <c r="C12" s="3">
+        <v>10.6</v>
+      </c>
+      <c r="D12" s="3">
+        <v>23.9</v>
+      </c>
+      <c r="E12" s="3">
+        <v>17.1</v>
+      </c>
+      <c r="F12" s="3">
+        <v>217</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrepiso vano extremo 1EC</t>
+          <t xml:space="preserve">Voladizo V 1.5 m</t>
         </is>
       </c>
       <c r="B13" s="3">
-        <v>4.75</v>
+        <v>1.27</v>
       </c>
       <c r="C13" s="3">
         <v>9.06</v>
       </c>
       <c r="D13" s="3">
-        <v>20.4</v>
-      </c>
-      <c r="E13" s="3">
-        <v>14.6</v>
+        <v>10.2</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
       </c>
       <c r="F13" s="3">
-        <v>185</v>
+        <v>152</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
@@ -1851,85 +2397,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cubierta vano 1EC (terraza L=5)</t>
-        </is>
-      </c>
-      <c r="B14" s="3">
-        <v>4.75</v>
-      </c>
-      <c r="C14" s="3">
-        <v>10.6</v>
-      </c>
-      <c r="D14" s="3">
-        <v>23.9</v>
-      </c>
-      <c r="E14" s="3">
-        <v>17.1</v>
-      </c>
-      <c r="F14" s="3">
-        <v>217</v>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 Nº4</t>
-        </is>
-      </c>
+      <c r="A14" s="0"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Voladizo V 1.5 m</t>
-        </is>
-      </c>
-      <c r="B15" s="3">
-        <v>1.27</v>
-      </c>
-      <c r="C15" s="3">
-        <v>9.06</v>
-      </c>
-      <c r="D15" s="3">
-        <v>10.2</v>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="F15" s="3">
-        <v>152</v>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 Nº4</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">CONCLUSIÓN</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aun con el coeficiente más exigente, As req (máx 217) &lt; 2 Nº4 (258) → gobierna acero mínimo (2 Nº4 sup. e inf.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cortante</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vu,máx 29.3 kN &lt; φ·1.1·Vc → no requiere estribos (C.8.3.3 permite +10% Vc en viguetas).</t>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aun con el coeficiente más exigente, As req &lt; 2 Nº4 → gobierna acero mínimo.</t>
         </is>
       </c>
     </row>
@@ -1940,408 +2418,318 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DISEÑO DE RIOSTRAS DE CIMENTACIÓN (VIGAS DE AMARRE)</t>
+          <t xml:space="preserve">DISEÑO DE RIOSTRAS DE CIMENTACIÓN (VIGAS DE AMARRE) — NSR-10 A.3.6.4.2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base: NSR-10 A.3.6.4.2 — el amarre resiste en tracción/compresión ≥ 0.25·Aa × carga vertical mayorada</t>
+          <t xml:space="preserve">El amarre resiste en tracción/compresión ≥ 0.25·Aa × carga vertical mayorada de la columna más cargada.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">de la columna más cargada que conecta.</t>
-        </is>
-      </c>
+      <c r="A3" s="0"/>
     </row>
     <row r="4">
-      <c r="A4" s="0"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N = 0.25·Aa·Pu</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.25·0.15·2591 kN</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">97.2 kN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FUERZA DE DISEÑO</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sección</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m (≥ ln/20)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d=232.6 mm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aa (Santa Marta)</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <v>0.15</v>
+          <t xml:space="preserve">Acero longitudinal</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5 simétrico (516 mm²)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">φAsfy=195 kN ≥ 97.2 OK</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pu máx columna (modelo SAP)</t>
+          <t xml:space="preserve">Estribos</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2591 kN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Nº3 @150 mm (@100 confinamiento)</t>
+        </is>
+      </c>
+      <c r="C7" s="5"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N = 0.25·Aa·Pu</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.25·0.15·2591</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">97.2 kN (tracc./compr.)</t>
-        </is>
-      </c>
+      <c r="A8" s="0"/>
     </row>
     <row r="9">
-      <c r="A9" s="0"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grupo</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longitud (m)</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº riostras*</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sección</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refuerzo</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SECCIÓN Y REFUERZO (uniforme, para la fuerza máxima)</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="B10" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C10" s="3">
+        <v>10</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dimensión mínima</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≥ ln/20 = 4000/20 = 200 mm</t>
+          <t xml:space="preserve">R-2</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <v>2.6</v>
+      </c>
+      <c r="C11" s="3">
+        <v>20</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sección adoptada</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30 × 0.30 m (d=232.6 mm)</t>
+          <t xml:space="preserve">R-3</t>
+        </is>
+      </c>
+      <c r="B12" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="C12" s="3">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">As por tracción</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N/(φ·fy)=97.2e3/(0.9·420)=257 mm²</t>
+          <t xml:space="preserve">R-4</t>
+        </is>
+      </c>
+      <c r="B13" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="C13" s="3">
+        <v>5</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">As mínimo (C.10.5)</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">233 mm²</t>
+          <t xml:space="preserve">R-5</t>
+        </is>
+      </c>
+      <c r="B14" s="3">
+        <v>3.65</v>
+      </c>
+      <c r="C14" s="3">
+        <v>10</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Refuerzo longitudinal</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5 simétrico (516 mm²) → φAsfy=195 kN ≥ 97.2 OK</t>
+          <t xml:space="preserve">R-6</t>
+        </is>
+      </c>
+      <c r="B15" s="3">
+        <v>3.85</v>
+      </c>
+      <c r="C15" s="3">
+        <v>26</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verif. compresión</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">φPn,máx=1220 kN &gt;&gt; 97.2 OK</t>
+          <t xml:space="preserve">R-7</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <v>3.9</v>
+      </c>
+      <c r="C16" s="3">
+        <v>26</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estribos</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº3 @150 mm; @100 mm confinamiento en extremos (2h)</t>
+          <t xml:space="preserve">R-8</t>
+        </is>
+      </c>
+      <c r="B17" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C17" s="3">
+        <v>10</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.30×0.30 m</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="0"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AGRUPACIÓN POR LONGITUD (despiece)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grupo</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Longitud (m)</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº riostras*</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sección</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Refuerzo</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-1</t>
-        </is>
-      </c>
-      <c r="B21" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="C21" s="3">
-        <v>10</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-2</t>
-        </is>
-      </c>
-      <c r="B22" s="3">
-        <v>2.6</v>
-      </c>
-      <c r="C22" s="3">
-        <v>20</v>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-3</t>
-        </is>
-      </c>
-      <c r="B23" s="3">
-        <v>2.7</v>
-      </c>
-      <c r="C23" s="3">
-        <v>5</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-4</t>
-        </is>
-      </c>
-      <c r="B24" s="3">
-        <v>2.8</v>
-      </c>
-      <c r="C24" s="3">
-        <v>5</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-5</t>
-        </is>
-      </c>
-      <c r="B25" s="3">
-        <v>3.65</v>
-      </c>
-      <c r="C25" s="3">
-        <v>10</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-6</t>
-        </is>
-      </c>
-      <c r="B26" s="3">
-        <v>3.85</v>
-      </c>
-      <c r="C26" s="3">
-        <v>26</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-7</t>
-        </is>
-      </c>
-      <c r="B27" s="3">
-        <v>3.9</v>
-      </c>
-      <c r="C27" s="3">
-        <v>26</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R-8</t>
-        </is>
-      </c>
-      <c r="B28" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="C28" s="3">
-        <v>10</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.30×0.30 m</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 Nº5</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">* Estimado para grilla 5 ejes X × 13 ejes Y; ajustar al plano de cimentación.</t>
-        </is>
-      </c>
-      <c r="B29" s="0"/>
-      <c r="C29" s="0"/>
-      <c r="D29" s="0"/>
-      <c r="E29" s="0"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">* Estimado para grilla 5×13 ejes; ajustar al plano de cimentación.</t>
+        </is>
+      </c>
+      <c r="B18" s="0"/>
+      <c r="C18" s="0"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>